<commit_message>
Finance : décisions D-21 à D-26 reportées dans les modèles, levée recalculée avec la love money (tranche 1 d'environ 70 000 €) (29/10/2026)
- Modèle Prévisions : sources et libellés mis à jour ; lignes 14 à 17 calculées à partir du calendrier des villes (D-25) ; love money de 70 000 € (D-26)
- Trésorerie, financement et tableau de bord recalculés : point bas de +10 071 € en mars 2027
- Note de levée : tranche 1 d'environ 70 000 € (45 000 € de BSA AIR), tranche 2 conditionnelle
- Fiche des données manquantes et README mis à jour

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2 FINANCE/FINANCEMENT/2026 1028 Modèle Pop Tables - Financement et table de capitalisation.xlsx
+++ b/2 FINANCE/FINANCEMENT/2026 1028 Modèle Pop Tables - Financement et table de capitalisation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vians\Documents\Claude\Projects\HEC-GEMM-Groupe-7\2 FINANCE\FINANCEMENT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{785A9667-D9AB-4BDC-966F-5B588B8F08AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B702530A-33A6-4C6D-8C33-D850546ABFBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{C6848D91-B8BF-4AD6-8B0B-F91FE7845E07}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="159">
   <si>
     <t>Financement — levées de fonds, prêts, subventions, table de capitalisation</t>
   </si>
@@ -375,15 +375,6 @@
     <t>État du fichier</t>
   </si>
   <si>
-    <t>[associés fondateurs, 7 membres de l'équipe]</t>
-  </si>
-  <si>
-    <t>Capital social de 7 000 € : 1 000 € par associé</t>
-  </si>
-  <si>
-    <t>Hypothèse temporaire ; nombre d'associés repris de README.md (sept fonctions, un responsable par fonction) ; montant à fixer par les associés</t>
-  </si>
-  <si>
     <t>[réseau d'accompagnement à la création]</t>
   </si>
   <si>
@@ -444,27 +435,45 @@
     <t>1 DIRECTION/STRATEGIE/2026 1027 Fiche de synthèse du projet, § Associé gastronomique (proposition)</t>
   </si>
   <si>
+    <t>Apport initial en love money (D-26)</t>
+  </si>
+  <si>
+    <t>[proches des fondateurs]</t>
+  </si>
+  <si>
+    <t>Décidé par la Direction le 29/10/2026 (D-26), aucun fonds versé ; forme à définir par le Juridique (capital, compte courant d'associés ou BSA AIR) ; non comptée dans la table de capitalisation tant que la forme n'est pas décidée</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>1 DIRECTION/STRATEGIE/2026 1029 Relevé de décisions du 29 octobre (matin), D-26</t>
+  </si>
+  <si>
     <t>Levée de fonds, tranche 1 (pré-amorçage)</t>
   </si>
   <si>
     <t>[business angels ; BSA AIR, sans valorisation fixée]</t>
   </si>
   <si>
-    <t>BSA AIR convertis lors d'une levée ultérieure, plafond de valorisation à négocier (P) ; à recevoir avant février 2027</t>
+    <t>D-23 (135 000 €) recalculée avec la love money : environ 70 000 € au total, dont 45 000 € de BSA AIR (P), à décider par la Direction ; à recevoir avant février 2027 ; plafond de valorisation à négocier</t>
   </si>
   <si>
     <t>P</t>
   </si>
   <si>
-    <t>2 FINANCE/FINANCEMENT/2026 1028 Note pour décision - levée de fonds Pop Tables, § 5</t>
-  </si>
-  <si>
-    <t>Levée de fonds, tranche 2 (conditionnelle)</t>
+    <t>2 FINANCE/FINANCEMENT/2026 1028 Note pour décision - levée de fonds Pop Tables, § 5 et 6</t>
+  </si>
+  <si>
+    <t>Levée de fonds, tranche 2 (conditionnelle, D-23)</t>
   </si>
   <si>
     <t>[business angels et investisseurs financiers, D-17]</t>
   </si>
   <si>
+    <t>Non nécessaire dans le plan. À décider en mai 2028 au vu des privatisations constatées, avant l'ouverture de 3 villes et 12 postes payés de plus (novembre 2028) : environ 215 000 € si elles restent proches de 8 par ville et par an (note, § 4)</t>
+  </si>
+  <si>
     <t>Idem</t>
   </si>
   <si>
@@ -480,7 +489,7 @@
     <t>Décision D-17 du 28/10/2026 ; part proposée dans l'onglet « Après levée »</t>
   </si>
   <si>
-    <t>Tranche 1 en BSA AIR (110 000 €), note pour décision du 28/10/2026 (soir) ; total à financer 135 000 €, dont 25 000 € de prêt d'honneur et de subvention. Calcul illustratif : les BSA AIR se convertiront au prix d'une levée ultérieure</t>
+    <t>Tranche 1 en BSA AIR (45 000 €), note pour décision recalculée le 29/10/2026 ; total à financer environ 70 000 €, dont 25 000 € de prêt d'honneur et de subvention. Calcul illustratif : les BSA AIR se convertiront au prix d'une levée ultérieure. La love money de 70 000 € (D-26) n'est pas comptée : si elle entre au capital, elle dilue aussi les fondateurs</t>
   </si>
   <si>
     <t>H non justifiée : aucune évaluation (voir la note pour décision du 28/10/2026, soir, § 5). À fonder sur les résultats des pilotes et de l'année 1</t>
@@ -504,16 +513,13 @@
     <t>Après levée : PROJECTION (pas un état)</t>
   </si>
   <si>
-    <t>Pop Tables (D-02 à D-20). Sources : 1 DIRECTION/STRATEGIE/2026 1028 Pop Tables - Cadre de référence et Business Model Canvas V5.</t>
-  </si>
-  <si>
-    <t>Mis à jour le 28/10/2026 (soir) : tranche 1 de 110 000 € en BSA AIR, tranche 2 conditionnelle (0 € dans le plan) et associé gastronomique en apport en industrie (D-17), selon la note pour décision du 28/10 (soir) et le budget revu par le responsable Finance. Aucun financement reçu ; tout reste au statut « Envisagé » (H ou P).</t>
+    <t>Pop Tables (D-02 à D-26). Sources : 1 DIRECTION/STRATEGIE/2026 1028 Pop Tables - Cadre de référence, Business Model Canvas V6 (D-24) et relevé du 29/10 (matin).</t>
+  </si>
+  <si>
+    <t>Mis à jour le 29/10/2026 : love money de 70 000 € (D-26) ; tranche 1 recalculée à environ 70 000 €, dont 45 000 € en BSA AIR (D-23 à confirmer par la Direction) ; tranche 2 conditionnelle (0 € dans le plan) ; associé gastronomique en apport en industrie (D-17). Aucun financement reçu ; tout reste au statut « Envisagé » (H ou P).</t>
   </si>
   <si>
     <t>Pop Tables · Pôle Finance · Version du 28/10/2026 (soir). Remplace le modèle du 27/10 (rangé dans 2 FINANCE/OLD).</t>
-  </si>
-  <si>
-    <t>Non nécessaire dans le plan. À décider en mai 2028 au vu des privatisations constatées, avant l'ouverture de 3 villes et 12 postes payés de plus (novembre 2028) : environ 220 000 € si elles restent proches de 8 par ville et par an (note, § 4)</t>
   </si>
 </sst>
 </file>
@@ -753,10 +759,10 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1106,7 +1112,7 @@
     </row>
     <row r="2" spans="1:2" ht="13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="13" x14ac:dyDescent="0.25">
@@ -1202,7 +1208,7 @@
         <v>23</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="13" x14ac:dyDescent="0.25">
@@ -1218,7 +1224,7 @@
         <v>109</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -1336,19 +1342,19 @@
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="62.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="100" x14ac:dyDescent="0.25">
       <c r="A6" s="7">
         <v>1</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>60</v>
+        <v>130</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>110</v>
+        <v>131</v>
       </c>
       <c r="D6" s="19"/>
       <c r="E6" s="20">
-        <v>7000</v>
+        <v>70000</v>
       </c>
       <c r="F6" s="18" t="s">
         <v>47</v>
@@ -1358,13 +1364,13 @@
       <c r="I6" s="19"/>
       <c r="J6" s="18"/>
       <c r="K6" s="18" t="s">
-        <v>111</v>
+        <v>132</v>
       </c>
       <c r="L6" s="18" t="s">
-        <v>49</v>
+        <v>133</v>
       </c>
       <c r="M6" s="18" t="s">
-        <v>112</v>
+        <v>134</v>
       </c>
       <c r="N6" s="18"/>
     </row>
@@ -1376,7 +1382,7 @@
         <v>43</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D7" s="19"/>
       <c r="E7" s="20">
@@ -1390,13 +1396,13 @@
       <c r="I7" s="19"/>
       <c r="J7" s="18"/>
       <c r="K7" s="18" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="L7" s="18" t="s">
         <v>49</v>
       </c>
       <c r="M7" s="18" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="N7" s="18"/>
     </row>
@@ -1408,7 +1414,7 @@
         <v>63</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D8" s="19"/>
       <c r="E8" s="20">
@@ -1422,29 +1428,29 @@
       <c r="I8" s="19"/>
       <c r="J8" s="18"/>
       <c r="K8" s="18" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="L8" s="18" t="s">
         <v>49</v>
       </c>
       <c r="M8" s="18" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="N8" s="18"/>
     </row>
-    <row r="9" spans="1:14" ht="50" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="75" x14ac:dyDescent="0.25">
       <c r="A9" s="7">
         <v>4</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D9" s="19"/>
       <c r="E9" s="20">
-        <v>110000</v>
+        <v>45000</v>
       </c>
       <c r="F9" s="18" t="s">
         <v>47</v>
@@ -1454,13 +1460,13 @@
       <c r="I9" s="19"/>
       <c r="J9" s="18"/>
       <c r="K9" s="18" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="L9" s="18" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="M9" s="18" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="N9" s="18"/>
     </row>
@@ -1469,10 +1475,10 @@
         <v>5</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D10" s="19"/>
       <c r="E10" s="20">
@@ -1486,13 +1492,13 @@
       <c r="I10" s="19"/>
       <c r="J10" s="18"/>
       <c r="K10" s="18" t="s">
-        <v>156</v>
+        <v>142</v>
       </c>
       <c r="L10" s="18" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="M10" s="18" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="N10" s="18"/>
     </row>
@@ -1501,10 +1507,10 @@
         <v>6</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D11" s="19"/>
       <c r="E11" s="20">
@@ -1518,13 +1524,13 @@
       <c r="I11" s="19"/>
       <c r="J11" s="18"/>
       <c r="K11" s="18" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="L11" s="18" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="M11" s="18" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="N11" s="18"/>
     </row>
@@ -1800,7 +1806,7 @@
       <c r="D28" s="2"/>
       <c r="E28" s="15">
         <f>SUMIFS(E6:E25,F6:F25,"&lt;&gt;Refusé")</f>
-        <v>142000</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="13" x14ac:dyDescent="0.3">
@@ -1865,7 +1871,7 @@
       </c>
       <c r="C35" s="13">
         <f t="shared" ref="C35:C41" si="0">SUMIFS($E$6:$E$25,$B$6:$B$25,B35,$F$6:$F$25,"&lt;&gt;Refusé")</f>
-        <v>7000</v>
+        <v>0</v>
       </c>
       <c r="D35" s="13">
         <f t="shared" ref="D35:D41" si="1">SUMIFS($H$6:$H$25,$B$6:$B$25,B35,$F$6:$F$25,"Fonds reçus")</f>
@@ -2042,7 +2048,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C5" s="10">
         <v>20000</v>
@@ -2063,13 +2069,13 @@
       </c>
       <c r="H5" s="9"/>
       <c r="I5" s="8" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="J5" s="8" t="s">
         <v>49</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -2320,13 +2326,13 @@
       <c r="C3" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="34" t="s">
-        <v>121</v>
-      </c>
-      <c r="E3" s="35"/>
-      <c r="F3" s="35"/>
-      <c r="G3" s="35"/>
-      <c r="H3" s="36"/>
+      <c r="D3" s="33" t="s">
+        <v>118</v>
+      </c>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="35"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
@@ -2362,10 +2368,10 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C6" s="22">
         <v>1000</v>
@@ -2385,10 +2391,10 @@
         <v>46327</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="J6" s="8" t="s">
         <v>49</v>
@@ -2396,10 +2402,10 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C7" s="22">
         <v>1000</v>
@@ -2419,10 +2425,10 @@
         <v>46327</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="J7" s="8" t="s">
         <v>49</v>
@@ -2430,10 +2436,10 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C8" s="22">
         <v>1000</v>
@@ -2453,10 +2459,10 @@
         <v>46327</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="J8" s="8" t="s">
         <v>49</v>
@@ -2464,10 +2470,10 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C9" s="22">
         <v>1000</v>
@@ -2487,10 +2493,10 @@
         <v>46327</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="J9" s="8" t="s">
         <v>49</v>
@@ -2498,10 +2504,10 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C10" s="22">
         <v>1000</v>
@@ -2521,10 +2527,10 @@
         <v>46327</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I10" s="8" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="J10" s="8" t="s">
         <v>49</v>
@@ -2532,10 +2538,10 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C11" s="22">
         <v>1000</v>
@@ -2555,10 +2561,10 @@
         <v>46327</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="J11" s="8" t="s">
         <v>49</v>
@@ -2566,10 +2572,10 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C12" s="22">
         <v>1000</v>
@@ -2589,10 +2595,10 @@
         <v>46327</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I12" s="8" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="J12" s="8" t="s">
         <v>49</v>
@@ -2751,7 +2757,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="13" x14ac:dyDescent="0.3">
@@ -2784,7 +2790,7 @@
         <v>49</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -2792,13 +2798,13 @@
         <v>97</v>
       </c>
       <c r="B6" s="10">
-        <v>110000</v>
+        <v>45000</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -2806,18 +2812,18 @@
         <v>98</v>
       </c>
       <c r="B7" s="29" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>49</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B8" s="31">
         <f>'Table de capitalisation'!C18+B26</f>
@@ -2839,7 +2845,7 @@
       </c>
       <c r="B10" s="14">
         <f>IF(B9&gt;0,ROUND(B6/B9,0),0)</f>
-        <v>2026</v>
+        <v>829</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -2848,7 +2854,7 @@
       </c>
       <c r="B11" s="13">
         <f>B5+B6</f>
-        <v>510000</v>
+        <v>445000</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -2857,21 +2863,21 @@
       </c>
       <c r="B12" s="26">
         <f>IF(B11&gt;0,B6/B11,0)</f>
-        <v>0.21568627450980393</v>
+        <v>0.10112359550561797</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="B13" s="33">
+        <v>151</v>
+      </c>
+      <c r="B13" s="36">
         <v>0.05</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2901,16 +2907,16 @@
         <v>1000</v>
       </c>
       <c r="C15" s="26">
-        <f t="shared" ref="C15:C25" si="0">IF($B$8=0,0,B15/$B$8)</f>
+        <f t="shared" ref="C15:C26" si="0">IF($B$8=0,0,B15/$B$8)</f>
         <v>0.13572204125950055</v>
       </c>
       <c r="D15" s="14">
-        <f t="shared" ref="D15:D25" si="1">B15</f>
+        <f t="shared" ref="D15:D26" si="1">B15</f>
         <v>1000</v>
       </c>
       <c r="E15" s="26">
         <f t="shared" ref="E15:E26" si="2">IF($D$28=0,0,D15/$D$28)</f>
-        <v>0.10645092612305727</v>
+        <v>0.12199585214102721</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -2932,7 +2938,7 @@
       </c>
       <c r="E16" s="26">
         <f t="shared" si="2"/>
-        <v>0.10645092612305727</v>
+        <v>0.12199585214102721</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -2954,7 +2960,7 @@
       </c>
       <c r="E17" s="26">
         <f t="shared" si="2"/>
-        <v>0.10645092612305727</v>
+        <v>0.12199585214102721</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -2976,7 +2982,7 @@
       </c>
       <c r="E18" s="26">
         <f t="shared" si="2"/>
-        <v>0.10645092612305727</v>
+        <v>0.12199585214102721</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -2998,7 +3004,7 @@
       </c>
       <c r="E19" s="26">
         <f t="shared" si="2"/>
-        <v>0.10645092612305727</v>
+        <v>0.12199585214102721</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -3020,7 +3026,7 @@
       </c>
       <c r="E20" s="26">
         <f t="shared" si="2"/>
-        <v>0.10645092612305727</v>
+        <v>0.12199585214102721</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -3042,7 +3048,7 @@
       </c>
       <c r="E21" s="26">
         <f t="shared" si="2"/>
-        <v>0.10645092612305727</v>
+        <v>0.12199585214102721</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -3135,7 +3141,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="30" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B26" s="31">
         <f>ROUND('Table de capitalisation'!C18*B13/(1-B13),0)</f>
@@ -3151,7 +3157,7 @@
       </c>
       <c r="E26" s="26">
         <f t="shared" si="2"/>
-        <v>3.9173940813285076E-2</v>
+        <v>4.4894473587898012E-2</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -3167,11 +3173,11 @@
       </c>
       <c r="D27" s="14">
         <f>B10</f>
-        <v>2026</v>
+        <v>829</v>
       </c>
       <c r="E27" s="26">
         <f>IF($D$28=0,0,D27/$D$28)</f>
-        <v>0.21566957632531403</v>
+        <v>0.10113456142491155</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="13" x14ac:dyDescent="0.3">
@@ -3188,11 +3194,11 @@
       </c>
       <c r="D28" s="16">
         <f>SUM(D15:D27)</f>
-        <v>9394</v>
+        <v>8197</v>
       </c>
       <c r="E28" s="27">
         <f>SUM(E15:E27)</f>
-        <v>1</v>
+        <v>0.99999999999999978</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="13" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Finance : SAS au capital de 70 000 € apporté à parts égales par les 7 fondateurs, sans BSA AIR ; table de capitalisation et note de levée mises à jour (29/10/2026)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2 FINANCE/FINANCEMENT/2026 1028 Modèle Pop Tables - Financement et table de capitalisation.xlsx
+++ b/2 FINANCE/FINANCEMENT/2026 1028 Modèle Pop Tables - Financement et table de capitalisation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vians\Documents\Claude\Projects\HEC-GEMM-Groupe-7\2 FINANCE\FINANCEMENT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B702530A-33A6-4C6D-8C33-D850546ABFBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECED950A-C313-44C3-9081-37566536AF70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{C6848D91-B8BF-4AD6-8B0B-F91FE7845E07}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="154">
   <si>
     <t>Financement — levées de fonds, prêts, subventions, table de capitalisation</t>
   </si>
@@ -399,9 +399,6 @@
     <t>Hypothèse temporaire (ligne 2 du suivi des financements)</t>
   </si>
   <si>
-    <t>Aucune : statuts non rédigés, société non créée (hypothèse temporaire)</t>
-  </si>
-  <si>
     <t>Associé fondateur (Direction)</t>
   </si>
   <si>
@@ -435,69 +432,21 @@
     <t>1 DIRECTION/STRATEGIE/2026 1027 Fiche de synthèse du projet, § Associé gastronomique (proposition)</t>
   </si>
   <si>
-    <t>Apport initial en love money (D-26)</t>
-  </si>
-  <si>
-    <t>[proches des fondateurs]</t>
-  </si>
-  <si>
-    <t>Décidé par la Direction le 29/10/2026 (D-26), aucun fonds versé ; forme à définir par le Juridique (capital, compte courant d'associés ou BSA AIR) ; non comptée dans la table de capitalisation tant que la forme n'est pas décidée</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>1 DIRECTION/STRATEGIE/2026 1029 Relevé de décisions du 29 octobre (matin), D-26</t>
-  </si>
-  <si>
-    <t>Levée de fonds, tranche 1 (pré-amorçage)</t>
-  </si>
-  <si>
-    <t>[business angels ; BSA AIR, sans valorisation fixée]</t>
-  </si>
-  <si>
-    <t>D-23 (135 000 €) recalculée avec la love money : environ 70 000 € au total, dont 45 000 € de BSA AIR (P), à décider par la Direction ; à recevoir avant février 2027 ; plafond de valorisation à négocier</t>
-  </si>
-  <si>
     <t>P</t>
   </si>
   <si>
     <t>2 FINANCE/FINANCEMENT/2026 1028 Note pour décision - levée de fonds Pop Tables, § 5 et 6</t>
   </si>
   <si>
-    <t>Levée de fonds, tranche 2 (conditionnelle, D-23)</t>
-  </si>
-  <si>
-    <t>[business angels et investisseurs financiers, D-17]</t>
-  </si>
-  <si>
-    <t>Non nécessaire dans le plan. À décider en mai 2028 au vu des privatisations constatées, avant l'ouverture de 3 villes et 12 postes payés de plus (novembre 2028) : environ 215 000 € si elles restent proches de 8 par ville et par an (note, § 4)</t>
-  </si>
-  <si>
     <t>Idem</t>
   </si>
   <si>
-    <t>Apport en industrie de l'associé gastronomique (D-17)</t>
-  </si>
-  <si>
     <t>[associé gastronomique, à identifier]</t>
   </si>
   <si>
-    <t>Actions en contrepartie de son réseau, de sa sélection et de son image ; aucune trésorerie ; forme à définir par le Juridique</t>
-  </si>
-  <si>
     <t>Décision D-17 du 28/10/2026 ; part proposée dans l'onglet « Après levée »</t>
   </si>
   <si>
-    <t>Tranche 1 en BSA AIR (45 000 €), note pour décision recalculée le 29/10/2026 ; total à financer environ 70 000 €, dont 25 000 € de prêt d'honneur et de subvention. Calcul illustratif : les BSA AIR se convertiront au prix d'une levée ultérieure. La love money de 70 000 € (D-26) n'est pas comptée : si elle entre au capital, elle dilue aussi les fondateurs</t>
-  </si>
-  <si>
-    <t>H non justifiée : aucune évaluation (voir la note pour décision du 28/10/2026, soir, § 5). À fonder sur les résultats des pilotes et de l'année 1</t>
-  </si>
-  <si>
-    <t>Business angels (BSA AIR, D-17)</t>
-  </si>
-  <si>
     <t>Part proposée pour l'associé gastronomique, avant la levée</t>
   </si>
   <si>
@@ -516,10 +465,46 @@
     <t>Pop Tables (D-02 à D-26). Sources : 1 DIRECTION/STRATEGIE/2026 1028 Pop Tables - Cadre de référence, Business Model Canvas V6 (D-24) et relevé du 29/10 (matin).</t>
   </si>
   <si>
-    <t>Mis à jour le 29/10/2026 : love money de 70 000 € (D-26) ; tranche 1 recalculée à environ 70 000 €, dont 45 000 € en BSA AIR (D-23 à confirmer par la Direction) ; tranche 2 conditionnelle (0 € dans le plan) ; associé gastronomique en apport en industrie (D-17). Aucun financement reçu ; tout reste au statut « Envisagé » (H ou P).</t>
-  </si>
-  <si>
     <t>Pop Tables · Pôle Finance · Version du 28/10/2026 (soir). Remplace le modèle du 27/10 (rangé dans 2 FINANCE/OLD).</t>
+  </si>
+  <si>
+    <t>Aucune : société non créée. Projet : SAS au capital de 70 000 €, 7 fondateurs à parts égales (10 000 actions de 1 € chacun), dont 2 fondateurs exécutifs ; choix du responsable Finance du 29/10/2026, statuts à rédiger par le Juridique</t>
+  </si>
+  <si>
+    <t>[7 fondateurs, à parts égales : 10 000 € chacun]</t>
+  </si>
+  <si>
+    <t>Capital initial de la SAS à sa création (novembre 2026) ; précise D-26 (mise de fonds de 70 000 €) : apport en capital des fondateurs, pas de BSA AIR. Aucun fonds versé</t>
+  </si>
+  <si>
+    <t>Choix du responsable Finance (29/10/2026) ; 1 DIRECTION/STRATEGIE/2026 1029 Relevé de décisions du 29 octobre (matin), D-26</t>
+  </si>
+  <si>
+    <t>[à décider : prêt bancaire ou apport complémentaire des fondateurs]</t>
+  </si>
+  <si>
+    <t>Complément de la réserve de l'année 1 (contingence et trésorerie de sécurité) ; remplace les 45 000 € de BSA AIR. Source à décider par la Direction</t>
+  </si>
+  <si>
+    <t>[augmentation de capital, investisseurs à identifier]</t>
+  </si>
+  <si>
+    <t>Tranche 2 conditionnelle (D-23) : non nécessaire dans le plan ; à décider en mai 2028 au vu des privatisations constatées. Environ 215 000 € si elles restent proches de 8 par ville et par an (note, § 4)</t>
+  </si>
+  <si>
+    <t>Apport en industrie (D-17) : actions en contrepartie de son réseau, de sa sélection et de son image ; aucune trésorerie ; forme à définir par le Juridique</t>
+  </si>
+  <si>
+    <t>Pas de levée en fonds propres dans le plan : pas de BSA AIR (choix du responsable Finance, 29/10/2026). Une augmentation de capital ne serait envisagée qu'en cas de tranche 2 (décision en mai 2028)</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>H non justifiée : aucune évaluation. Ne sert qu'en cas d'augmentation de capital (tranche 2)</t>
+  </si>
+  <si>
+    <t>Mis à jour le 29/10/2026 : SAS au capital de 70 000 €, apporté à parts égales par les 7 fondateurs (D-26, forme précisée par le responsable Finance) ; pas de BSA AIR ; complément de 45 000 € à décider (prêt bancaire ou apport complémentaire) ; tranche 2 conditionnelle en augmentation de capital ; associé gastronomique en apport en industrie (D-17). Aucun financement reçu ; tout reste au statut « Envisagé ».</t>
   </si>
 </sst>
 </file>
@@ -759,10 +744,10 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1112,7 +1097,7 @@
     </row>
     <row r="2" spans="1:2" ht="13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>158</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="13" x14ac:dyDescent="0.25">
@@ -1208,7 +1193,7 @@
         <v>23</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>156</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="13" x14ac:dyDescent="0.25">
@@ -1219,12 +1204,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="50" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>109</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -1342,15 +1327,15 @@
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="100" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="62.5" x14ac:dyDescent="0.25">
       <c r="A6" s="7">
         <v>1</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>130</v>
+        <v>60</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="D6" s="19"/>
       <c r="E6" s="20">
@@ -1364,13 +1349,13 @@
       <c r="I6" s="19"/>
       <c r="J6" s="18"/>
       <c r="K6" s="18" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="L6" s="18" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="M6" s="18" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="N6" s="18"/>
     </row>
@@ -1438,15 +1423,15 @@
       </c>
       <c r="N8" s="18"/>
     </row>
-    <row r="9" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="62.5" x14ac:dyDescent="0.25">
       <c r="A9" s="7">
         <v>4</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>135</v>
+        <v>65</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="D9" s="19"/>
       <c r="E9" s="20">
@@ -1460,25 +1445,25 @@
       <c r="I9" s="19"/>
       <c r="J9" s="18"/>
       <c r="K9" s="18" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="L9" s="18" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="M9" s="18" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="N9" s="18"/>
     </row>
-    <row r="10" spans="1:14" ht="100" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" ht="75" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
         <v>5</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>140</v>
+        <v>61</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="D10" s="19"/>
       <c r="E10" s="20">
@@ -1492,25 +1477,25 @@
       <c r="I10" s="19"/>
       <c r="J10" s="18"/>
       <c r="K10" s="18" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="L10" s="18" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="M10" s="18" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="N10" s="18"/>
     </row>
-    <row r="11" spans="1:14" ht="50" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" ht="62.5" x14ac:dyDescent="0.25">
       <c r="A11" s="7">
         <v>6</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>144</v>
+        <v>60</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="D11" s="19"/>
       <c r="E11" s="20">
@@ -1524,13 +1509,13 @@
       <c r="I11" s="19"/>
       <c r="J11" s="18"/>
       <c r="K11" s="18" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="L11" s="18" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="M11" s="18" t="s">
-        <v>147</v>
+        <v>133</v>
       </c>
       <c r="N11" s="18"/>
     </row>
@@ -1871,7 +1856,7 @@
       </c>
       <c r="C35" s="13">
         <f t="shared" ref="C35:C41" si="0">SUMIFS($E$6:$E$25,$B$6:$B$25,B35,$F$6:$F$25,"&lt;&gt;Refusé")</f>
-        <v>0</v>
+        <v>70000</v>
       </c>
       <c r="D35" s="13">
         <f t="shared" ref="D35:D41" si="1">SUMIFS($H$6:$H$25,$B$6:$B$25,B35,$F$6:$F$25,"Fonds reçus")</f>
@@ -1949,7 +1934,7 @@
       </c>
       <c r="C41" s="13">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>45000</v>
       </c>
       <c r="D41" s="13">
         <f t="shared" si="1"/>
@@ -2326,13 +2311,13 @@
       <c r="C3" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="D3" s="33" t="s">
-        <v>118</v>
-      </c>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="35"/>
+      <c r="D3" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="36"/>
     </row>
     <row r="5" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
@@ -2368,13 +2353,13 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>120</v>
-      </c>
       <c r="C6" s="22">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="D6" s="26">
         <f t="shared" ref="D6:D17" si="0">IF(OR(B6="BSA ou BSPCE non exercés",$C$18-$C$19=0),0,C6/($C$18-$C$19))</f>
@@ -2385,30 +2370,30 @@
         <v>0.14285714285714285</v>
       </c>
       <c r="F6" s="10">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="G6" s="9">
         <v>46327</v>
       </c>
       <c r="H6" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="I6" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="I6" s="8" t="s">
-        <v>122</v>
-      </c>
       <c r="J6" s="8" t="s">
-        <v>49</v>
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C7" s="22">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="D7" s="26">
         <f t="shared" si="0"/>
@@ -2419,30 +2404,30 @@
         <v>0.14285714285714285</v>
       </c>
       <c r="F7" s="10">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="G7" s="9">
         <v>46327</v>
       </c>
       <c r="H7" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="I7" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="I7" s="8" t="s">
-        <v>122</v>
-      </c>
       <c r="J7" s="8" t="s">
-        <v>49</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C8" s="22">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="D8" s="26">
         <f t="shared" si="0"/>
@@ -2453,30 +2438,30 @@
         <v>0.14285714285714285</v>
       </c>
       <c r="F8" s="10">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="G8" s="9">
         <v>46327</v>
       </c>
       <c r="H8" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="I8" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="I8" s="8" t="s">
-        <v>122</v>
-      </c>
       <c r="J8" s="8" t="s">
-        <v>49</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C9" s="22">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="D9" s="26">
         <f t="shared" si="0"/>
@@ -2487,30 +2472,30 @@
         <v>0.14285714285714285</v>
       </c>
       <c r="F9" s="10">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="G9" s="9">
         <v>46327</v>
       </c>
       <c r="H9" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="I9" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="I9" s="8" t="s">
-        <v>122</v>
-      </c>
       <c r="J9" s="8" t="s">
-        <v>49</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C10" s="22">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="D10" s="26">
         <f t="shared" si="0"/>
@@ -2521,30 +2506,30 @@
         <v>0.14285714285714285</v>
       </c>
       <c r="F10" s="10">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="G10" s="9">
         <v>46327</v>
       </c>
       <c r="H10" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="I10" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="I10" s="8" t="s">
-        <v>122</v>
-      </c>
       <c r="J10" s="8" t="s">
-        <v>49</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C11" s="22">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="D11" s="26">
         <f t="shared" si="0"/>
@@ -2555,30 +2540,30 @@
         <v>0.14285714285714285</v>
       </c>
       <c r="F11" s="10">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="G11" s="9">
         <v>46327</v>
       </c>
       <c r="H11" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="I11" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="I11" s="8" t="s">
-        <v>122</v>
-      </c>
       <c r="J11" s="8" t="s">
-        <v>49</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C12" s="22">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="D12" s="26">
         <f t="shared" si="0"/>
@@ -2589,19 +2574,19 @@
         <v>0.14285714285714285</v>
       </c>
       <c r="F12" s="10">
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="G12" s="9">
         <v>46327</v>
       </c>
       <c r="H12" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="I12" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="I12" s="8" t="s">
-        <v>122</v>
-      </c>
       <c r="J12" s="8" t="s">
-        <v>49</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -2701,7 +2686,7 @@
       <c r="B18" s="2"/>
       <c r="C18" s="16">
         <f>SUM(C6:C17)</f>
-        <v>7000</v>
+        <v>70000</v>
       </c>
       <c r="D18" s="27">
         <f>SUM(D6:D17)</f>
@@ -2713,7 +2698,7 @@
       </c>
       <c r="F18" s="15">
         <f>SUM(F6:F17)</f>
-        <v>7000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="13" x14ac:dyDescent="0.3">
@@ -2757,7 +2742,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>155</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="13" x14ac:dyDescent="0.3">
@@ -2790,7 +2775,7 @@
         <v>49</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -2798,13 +2783,13 @@
         <v>97</v>
       </c>
       <c r="B6" s="10">
-        <v>45000</v>
+        <v>0</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -2812,22 +2797,22 @@
         <v>98</v>
       </c>
       <c r="B7" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>49</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>154</v>
+        <v>137</v>
       </c>
       <c r="B8" s="31">
         <f>'Table de capitalisation'!C18+B26</f>
-        <v>7368</v>
+        <v>73684</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -2836,7 +2821,7 @@
       </c>
       <c r="B9" s="23">
         <f>IF(B8&gt;0,B5/B8,0)</f>
-        <v>54.28881650380022</v>
+        <v>5.4285869388198256</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -2845,7 +2830,7 @@
       </c>
       <c r="B10" s="14">
         <f>IF(B9&gt;0,ROUND(B6/B9,0),0)</f>
-        <v>829</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -2854,7 +2839,7 @@
       </c>
       <c r="B11" s="13">
         <f>B5+B6</f>
-        <v>445000</v>
+        <v>400000</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -2863,21 +2848,21 @@
       </c>
       <c r="B12" s="26">
         <f>IF(B11&gt;0,B6/B11,0)</f>
-        <v>0.10112359550561797</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="B13" s="36">
+        <v>134</v>
+      </c>
+      <c r="B13" s="33">
         <v>0.05</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2904,19 +2889,19 @@
       </c>
       <c r="B15" s="31">
         <f>'Table de capitalisation'!C6</f>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="C15" s="26">
-        <f t="shared" ref="C15:C26" si="0">IF($B$8=0,0,B15/$B$8)</f>
-        <v>0.13572204125950055</v>
+        <f t="shared" ref="C15:C25" si="0">IF($B$8=0,0,B15/$B$8)</f>
+        <v>0.13571467347049562</v>
       </c>
       <c r="D15" s="14">
-        <f t="shared" ref="D15:D26" si="1">B15</f>
-        <v>1000</v>
+        <f t="shared" ref="D15:D25" si="1">B15</f>
+        <v>10000</v>
       </c>
       <c r="E15" s="26">
         <f t="shared" ref="E15:E26" si="2">IF($D$28=0,0,D15/$D$28)</f>
-        <v>0.12199585214102721</v>
+        <v>0.13571467347049562</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -2926,19 +2911,19 @@
       </c>
       <c r="B16" s="31">
         <f>'Table de capitalisation'!C7</f>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="C16" s="26">
         <f t="shared" si="0"/>
-        <v>0.13572204125950055</v>
+        <v>0.13571467347049562</v>
       </c>
       <c r="D16" s="14">
         <f t="shared" si="1"/>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="E16" s="26">
         <f t="shared" si="2"/>
-        <v>0.12199585214102721</v>
+        <v>0.13571467347049562</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -2948,19 +2933,19 @@
       </c>
       <c r="B17" s="31">
         <f>'Table de capitalisation'!C8</f>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="C17" s="26">
         <f t="shared" si="0"/>
-        <v>0.13572204125950055</v>
+        <v>0.13571467347049562</v>
       </c>
       <c r="D17" s="14">
         <f t="shared" si="1"/>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="E17" s="26">
         <f t="shared" si="2"/>
-        <v>0.12199585214102721</v>
+        <v>0.13571467347049562</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -2970,19 +2955,19 @@
       </c>
       <c r="B18" s="31">
         <f>'Table de capitalisation'!C9</f>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="C18" s="26">
         <f t="shared" si="0"/>
-        <v>0.13572204125950055</v>
+        <v>0.13571467347049562</v>
       </c>
       <c r="D18" s="14">
         <f t="shared" si="1"/>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="E18" s="26">
         <f t="shared" si="2"/>
-        <v>0.12199585214102721</v>
+        <v>0.13571467347049562</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -2992,19 +2977,19 @@
       </c>
       <c r="B19" s="31">
         <f>'Table de capitalisation'!C10</f>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="C19" s="26">
         <f t="shared" si="0"/>
-        <v>0.13572204125950055</v>
+        <v>0.13571467347049562</v>
       </c>
       <c r="D19" s="14">
         <f t="shared" si="1"/>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="E19" s="26">
         <f t="shared" si="2"/>
-        <v>0.12199585214102721</v>
+        <v>0.13571467347049562</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -3014,19 +2999,19 @@
       </c>
       <c r="B20" s="31">
         <f>'Table de capitalisation'!C11</f>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="C20" s="26">
         <f t="shared" si="0"/>
-        <v>0.13572204125950055</v>
+        <v>0.13571467347049562</v>
       </c>
       <c r="D20" s="14">
         <f t="shared" si="1"/>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="E20" s="26">
         <f t="shared" si="2"/>
-        <v>0.12199585214102721</v>
+        <v>0.13571467347049562</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -3036,19 +3021,19 @@
       </c>
       <c r="B21" s="31">
         <f>'Table de capitalisation'!C12</f>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="C21" s="26">
         <f t="shared" si="0"/>
-        <v>0.13572204125950055</v>
+        <v>0.13571467347049562</v>
       </c>
       <c r="D21" s="14">
         <f t="shared" si="1"/>
-        <v>1000</v>
+        <v>10000</v>
       </c>
       <c r="E21" s="26">
         <f t="shared" si="2"/>
-        <v>0.12199585214102721</v>
+        <v>0.13571467347049562</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -3141,29 +3126,29 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="30" t="s">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="B26" s="31">
         <f>ROUND('Table de capitalisation'!C18*B13/(1-B13),0)</f>
-        <v>368</v>
+        <v>3684</v>
       </c>
       <c r="C26" s="26">
         <f>IF($B$8=0,0,B26/$B$8)</f>
-        <v>4.9945711183496201E-2</v>
+        <v>4.9997285706530593E-2</v>
       </c>
       <c r="D26" s="14">
         <f>B26</f>
-        <v>368</v>
+        <v>3684</v>
       </c>
       <c r="E26" s="26">
         <f t="shared" si="2"/>
-        <v>4.4894473587898012E-2</v>
+        <v>4.9997285706530593E-2</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="str">
         <f>IF(B7="","Nouveaux investisseurs",B7)</f>
-        <v>Business angels (BSA AIR, D-17)</v>
+        <v>Nouveaux investisseurs</v>
       </c>
       <c r="B27" s="14">
         <v>0</v>
@@ -3173,11 +3158,11 @@
       </c>
       <c r="D27" s="14">
         <f>B10</f>
-        <v>829</v>
+        <v>0</v>
       </c>
       <c r="E27" s="26">
         <f>IF($D$28=0,0,D27/$D$28)</f>
-        <v>0.10113456142491155</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="13" x14ac:dyDescent="0.3">
@@ -3186,19 +3171,19 @@
       </c>
       <c r="B28" s="16">
         <f>SUM(B15:B27)</f>
-        <v>7368</v>
+        <v>73684</v>
       </c>
       <c r="C28" s="27">
         <f>SUM(C15:C27)</f>
-        <v>1.0000000000000002</v>
+        <v>0.99999999999999989</v>
       </c>
       <c r="D28" s="16">
         <f>SUM(D15:D27)</f>
-        <v>8197</v>
+        <v>73684</v>
       </c>
       <c r="E28" s="27">
         <f>SUM(E15:E27)</f>
-        <v>0.99999999999999978</v>
+        <v>0.99999999999999989</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="13" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Finance : financement exclusivement par l'apport des 7 fondateurs, note de levée rangée dans OLD ; pitch, partie 7 « Finance » (29/10/2026)
- Modèle Financement : prêt d'honneur, subvention, complément et tranche 2 retirés ; seul reste le capital de 70 000 €
- Note pour décision sur la levée de fonds rangée dans 2 FINANCE/OLD
- Fiche des données manquantes et README mis à jour
- Slide de synthèse Finance du pitch (origine des fonds, CA et résultat par an, valorisation à 3 ans) déposée dans TRAVAUX

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2 FINANCE/FINANCEMENT/2026 1028 Modèle Pop Tables - Financement et table de capitalisation.xlsx
+++ b/2 FINANCE/FINANCEMENT/2026 1028 Modèle Pop Tables - Financement et table de capitalisation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vians\Documents\Claude\Projects\HEC-GEMM-Groupe-7\2 FINANCE\FINANCEMENT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECED950A-C313-44C3-9081-37566536AF70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{922FDB80-5A7B-47FC-A90E-F0C16B2DBD9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{C6848D91-B8BF-4AD6-8B0B-F91FE7845E07}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="19200" windowHeight="9970" xr2:uid="{C6848D91-B8BF-4AD6-8B0B-F91FE7845E07}"/>
   </bookViews>
   <sheets>
     <sheet name="Mode d'emploi" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="140">
   <si>
     <t>Financement — levées de fonds, prêts, subventions, table de capitalisation</t>
   </si>
@@ -375,30 +375,6 @@
     <t>État du fichier</t>
   </si>
   <si>
-    <t>[réseau d'accompagnement à la création]</t>
-  </si>
-  <si>
-    <t>Prêt personnel aux fondateurs, taux zéro, 5 ans (H)</t>
-  </si>
-  <si>
-    <t>Hypothèse temporaire ; couvre le besoin de l'année 1 du plan financier (2 FINANCE/PREVISIONS)</t>
-  </si>
-  <si>
-    <t>[concours ou incubateur]</t>
-  </si>
-  <si>
-    <t>À identifier</t>
-  </si>
-  <si>
-    <t>Hypothèse temporaire ; aucun dispositif identifié dans le dépôt</t>
-  </si>
-  <si>
-    <t>Aucune : prêt non signé, simulation</t>
-  </si>
-  <si>
-    <t>Hypothèse temporaire (ligne 2 du suivi des financements)</t>
-  </si>
-  <si>
     <t>Associé fondateur (Direction)</t>
   </si>
   <si>
@@ -435,12 +411,6 @@
     <t>P</t>
   </si>
   <si>
-    <t>2 FINANCE/FINANCEMENT/2026 1028 Note pour décision - levée de fonds Pop Tables, § 5 et 6</t>
-  </si>
-  <si>
-    <t>Idem</t>
-  </si>
-  <si>
     <t>[associé gastronomique, à identifier]</t>
   </si>
   <si>
@@ -474,37 +444,25 @@
     <t>[7 fondateurs, à parts égales : 10 000 € chacun]</t>
   </si>
   <si>
-    <t>Capital initial de la SAS à sa création (novembre 2026) ; précise D-26 (mise de fonds de 70 000 €) : apport en capital des fondateurs, pas de BSA AIR. Aucun fonds versé</t>
-  </si>
-  <si>
     <t>Choix du responsable Finance (29/10/2026) ; 1 DIRECTION/STRATEGIE/2026 1029 Relevé de décisions du 29 octobre (matin), D-26</t>
   </si>
   <si>
-    <t>[à décider : prêt bancaire ou apport complémentaire des fondateurs]</t>
-  </si>
-  <si>
-    <t>Complément de la réserve de l'année 1 (contingence et trésorerie de sécurité) ; remplace les 45 000 € de BSA AIR. Source à décider par la Direction</t>
-  </si>
-  <si>
-    <t>[augmentation de capital, investisseurs à identifier]</t>
-  </si>
-  <si>
-    <t>Tranche 2 conditionnelle (D-23) : non nécessaire dans le plan ; à décider en mai 2028 au vu des privatisations constatées. Environ 215 000 € si elles restent proches de 8 par ville et par an (note, § 4)</t>
-  </si>
-  <si>
     <t>Apport en industrie (D-17) : actions en contrepartie de son réseau, de sa sélection et de son image ; aucune trésorerie ; forme à définir par le Juridique</t>
   </si>
   <si>
-    <t>Pas de levée en fonds propres dans le plan : pas de BSA AIR (choix du responsable Finance, 29/10/2026). Une augmentation de capital ne serait envisagée qu'en cas de tranche 2 (décision en mai 2028)</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
-    <t>H non justifiée : aucune évaluation. Ne sert qu'en cas d'augmentation de capital (tranche 2)</t>
-  </si>
-  <si>
-    <t>Mis à jour le 29/10/2026 : SAS au capital de 70 000 €, apporté à parts égales par les 7 fondateurs (D-26, forme précisée par le responsable Finance) ; pas de BSA AIR ; complément de 45 000 € à décider (prêt bancaire ou apport complémentaire) ; tranche 2 conditionnelle en augmentation de capital ; associé gastronomique en apport en industrie (D-17). Aucun financement reçu ; tout reste au statut « Envisagé ».</t>
+    <t>Capital initial de la SAS à sa création (novembre 2026) ; seule source de financement du plan (choix du responsable Finance, 29/10/2026, conforme au budget sur 36 mois) : ni prêt, ni subvention, ni levée. Précise D-26. Aucun fonds versé</t>
+  </si>
+  <si>
+    <t>Aucune levée prévue : le plan est financé exclusivement par l'apport des 7 fondateurs (choix du responsable Finance, 29/10/2026). Onglet conservé pour simuler une éventuelle augmentation de capital future</t>
+  </si>
+  <si>
+    <t>H non justifiée : aucune évaluation. Ne sert qu'en cas d'augmentation de capital future</t>
+  </si>
+  <si>
+    <t>Mis à jour le 29/10/2026 : financement exclusivement par l'apport des 7 fondateurs, à parts égales (SAS au capital de 70 000 €, D-26), conformément au budget sur 36 mois. Ni prêt d'honneur, ni subvention, ni levée de fonds. Associé gastronomique en apport en industrie (D-17), sans trésorerie. Aucun fonds versé ; tout reste au statut « Envisagé ».</t>
   </si>
 </sst>
 </file>
@@ -1097,7 +1055,7 @@
     </row>
     <row r="2" spans="1:2" ht="13" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="13" x14ac:dyDescent="0.25">
@@ -1193,7 +1151,7 @@
         <v>23</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="13" x14ac:dyDescent="0.25">
@@ -1204,12 +1162,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="50" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>109</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -1327,7 +1285,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="62.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" ht="87.5" x14ac:dyDescent="0.25">
       <c r="A6" s="7">
         <v>1</v>
       </c>
@@ -1335,7 +1293,7 @@
         <v>60</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="D6" s="19"/>
       <c r="E6" s="20">
@@ -1349,142 +1307,86 @@
       <c r="I6" s="19"/>
       <c r="J6" s="18"/>
       <c r="K6" s="18" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="L6" s="18" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="M6" s="18" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="N6" s="18"/>
     </row>
-    <row r="7" spans="1:14" ht="37.5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="7">
         <v>2</v>
       </c>
-      <c r="B7" s="18" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>110</v>
-      </c>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
       <c r="D7" s="19"/>
-      <c r="E7" s="20">
-        <v>20000</v>
-      </c>
-      <c r="F7" s="18" t="s">
-        <v>47</v>
-      </c>
+      <c r="E7" s="20"/>
+      <c r="F7" s="18"/>
       <c r="G7" s="20"/>
       <c r="H7" s="20"/>
       <c r="I7" s="19"/>
       <c r="J7" s="18"/>
-      <c r="K7" s="18" t="s">
-        <v>111</v>
-      </c>
-      <c r="L7" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="M7" s="18" t="s">
-        <v>112</v>
-      </c>
+      <c r="K7" s="18"/>
+      <c r="L7" s="18"/>
+      <c r="M7" s="18"/>
       <c r="N7" s="18"/>
     </row>
-    <row r="8" spans="1:14" ht="25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
         <v>3</v>
       </c>
-      <c r="B8" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>113</v>
-      </c>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
       <c r="D8" s="19"/>
-      <c r="E8" s="20">
-        <v>5000</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>47</v>
-      </c>
+      <c r="E8" s="20"/>
+      <c r="F8" s="18"/>
       <c r="G8" s="20"/>
       <c r="H8" s="20"/>
       <c r="I8" s="19"/>
       <c r="J8" s="18"/>
-      <c r="K8" s="18" t="s">
-        <v>114</v>
-      </c>
-      <c r="L8" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="M8" s="18" t="s">
-        <v>115</v>
-      </c>
+      <c r="K8" s="18"/>
+      <c r="L8" s="18"/>
+      <c r="M8" s="18"/>
       <c r="N8" s="18"/>
     </row>
-    <row r="9" spans="1:14" ht="62.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="7">
         <v>4</v>
       </c>
-      <c r="B9" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>145</v>
-      </c>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
       <c r="D9" s="19"/>
-      <c r="E9" s="20">
-        <v>45000</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>47</v>
-      </c>
+      <c r="E9" s="20"/>
+      <c r="F9" s="18"/>
       <c r="G9" s="20"/>
       <c r="H9" s="20"/>
       <c r="I9" s="19"/>
       <c r="J9" s="18"/>
-      <c r="K9" s="18" t="s">
-        <v>146</v>
-      </c>
-      <c r="L9" s="18" t="s">
-        <v>129</v>
-      </c>
-      <c r="M9" s="18" t="s">
-        <v>130</v>
-      </c>
+      <c r="K9" s="18"/>
+      <c r="L9" s="18"/>
+      <c r="M9" s="18"/>
       <c r="N9" s="18"/>
     </row>
-    <row r="10" spans="1:14" ht="75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
         <v>5</v>
       </c>
-      <c r="B10" s="18" t="s">
-        <v>61</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>147</v>
-      </c>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
       <c r="D10" s="19"/>
-      <c r="E10" s="20">
-        <v>0</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>47</v>
-      </c>
+      <c r="E10" s="20"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="20"/>
       <c r="H10" s="20"/>
       <c r="I10" s="19"/>
       <c r="J10" s="18"/>
-      <c r="K10" s="18" t="s">
-        <v>148</v>
-      </c>
-      <c r="L10" s="18" t="s">
-        <v>129</v>
-      </c>
-      <c r="M10" s="18" t="s">
-        <v>131</v>
-      </c>
+      <c r="K10" s="18"/>
+      <c r="L10" s="18"/>
+      <c r="M10" s="18"/>
       <c r="N10" s="18"/>
     </row>
     <row r="11" spans="1:14" ht="62.5" x14ac:dyDescent="0.25">
@@ -1495,7 +1397,7 @@
         <v>60</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="D11" s="19"/>
       <c r="E11" s="20">
@@ -1509,13 +1411,13 @@
       <c r="I11" s="19"/>
       <c r="J11" s="18"/>
       <c r="K11" s="18" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="L11" s="18" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="M11" s="18" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="N11" s="18"/>
     </row>
@@ -1791,7 +1693,7 @@
       <c r="D28" s="2"/>
       <c r="E28" s="15">
         <f>SUMIFS(E6:E25,F6:F25,"&lt;&gt;Refusé")</f>
-        <v>140000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="13" x14ac:dyDescent="0.3">
@@ -1895,7 +1797,7 @@
       </c>
       <c r="C38" s="13">
         <f t="shared" si="0"/>
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="D38" s="13">
         <f t="shared" si="1"/>
@@ -1908,7 +1810,7 @@
       </c>
       <c r="C39" s="13">
         <f t="shared" si="0"/>
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="D39" s="13">
         <f t="shared" si="1"/>
@@ -1934,7 +1836,7 @@
       </c>
       <c r="C41" s="13">
         <f t="shared" si="0"/>
-        <v>45000</v>
+        <v>0</v>
       </c>
       <c r="D41" s="13">
         <f t="shared" si="1"/>
@@ -2029,39 +1931,23 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="8">
-        <v>2</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="C5" s="10">
-        <v>20000</v>
-      </c>
-      <c r="D5" s="21">
-        <v>0</v>
-      </c>
-      <c r="E5" s="22">
-        <v>60</v>
-      </c>
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="22"/>
       <c r="F5" s="23">
         <f t="shared" ref="F5:F14" si="0">IF(AND(C5&gt;0,E5&gt;0),IF(D5=0,C5/E5,PMT(D5/12,E5,-C5)),0)</f>
-        <v>333.33333333333331</v>
+        <v>0</v>
       </c>
       <c r="G5" s="23">
         <f t="shared" ref="G5:G14" si="1">IF(F5&gt;0,F5*E5-C5,0)</f>
         <v>0</v>
       </c>
       <c r="H5" s="9"/>
-      <c r="I5" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="K5" s="8" t="s">
-        <v>117</v>
-      </c>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="8"/>
@@ -2241,13 +2127,13 @@
       </c>
       <c r="C15" s="15">
         <f>SUM(C5:C14)</f>
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="24">
         <f>SUM(F5:F14)</f>
-        <v>333.33333333333331</v>
+        <v>0</v>
       </c>
       <c r="G15" s="24">
         <f>SUM(G5:G14)</f>
@@ -2312,7 +2198,7 @@
         <v>82</v>
       </c>
       <c r="D3" s="34" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="E3" s="35"/>
       <c r="F3" s="35"/>
@@ -2353,10 +2239,10 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C6" s="22">
         <v>10000</v>
@@ -2376,21 +2262,21 @@
         <v>46327</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="I6" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="J6" s="8" t="s">
         <v>121</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C7" s="22">
         <v>10000</v>
@@ -2410,21 +2296,21 @@
         <v>46327</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="I7" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="J7" s="8" t="s">
         <v>121</v>
-      </c>
-      <c r="J7" s="8" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C8" s="22">
         <v>10000</v>
@@ -2444,21 +2330,21 @@
         <v>46327</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="I8" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="J8" s="8" t="s">
         <v>121</v>
-      </c>
-      <c r="J8" s="8" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C9" s="22">
         <v>10000</v>
@@ -2478,21 +2364,21 @@
         <v>46327</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="I9" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="J9" s="8" t="s">
         <v>121</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C10" s="22">
         <v>10000</v>
@@ -2512,21 +2398,21 @@
         <v>46327</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="I10" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="J10" s="8" t="s">
         <v>121</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C11" s="22">
         <v>10000</v>
@@ -2546,21 +2432,21 @@
         <v>46327</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="I11" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="J11" s="8" t="s">
         <v>121</v>
-      </c>
-      <c r="J11" s="8" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="C12" s="22">
         <v>10000</v>
@@ -2580,13 +2466,13 @@
         <v>46327</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="I12" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="J12" s="8" t="s">
         <v>121</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -2742,7 +2628,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="13" x14ac:dyDescent="0.3">
@@ -2775,7 +2661,7 @@
         <v>49</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -2786,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -2797,18 +2683,18 @@
         <v>98</v>
       </c>
       <c r="B7" s="29" t="s">
-        <v>151</v>
+        <v>135</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>49</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="B8" s="31">
         <f>'Table de capitalisation'!C18+B26</f>
@@ -2853,16 +2739,16 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="B13" s="33">
         <v>0.05</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3126,7 +3012,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="30" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="B26" s="31">
         <f>ROUND('Table de capitalisation'!C18*B13/(1-B13),0)</f>

</xml_diff>